<commit_message>
ANS-009-011 - Retours sur la partie sécurité et signature (#39)
* Correction des premiers retour sur la section sécurité / imputabilité: 1/correction du paragraphe introductif ; 2/ correction de la partie confidentialité

* corrections des coquilles visuelles et structures du markdown

* Correction section sécurité (2) : 1/Reformulation de la section Imputabilité, 2/ retrait des mentions PGSSI-S, 3/ ajout d'un paragraphe Tracabilité

* Rajout du terme "PGSSI-S" qui a été supprimée dans la partie introductive lors du commit 398187cb4a6431e5e1e05e2ca5273006e3986a79 362ec5f76a50d32992af1cb948283f37854cc8a4
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-xdmAuthor.xlsx
+++ b/main/ig/StructureDefinition-xdmAuthor.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-07T08:39:35+00:00</t>
+    <t>2026-09-30T09:03:39+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -307,7 +307,7 @@
     <t>**AutorSpecialty**</t>
   </si>
   <si>
-    <t>https://mos.esante.gouv.fr/NOS/JDV_J01-XdsAuthorSpecialty-CISIS/FHIR/JDV-J01-XdsAuthorSpecialty-CISIS|20260505120000</t>
+    <t>https://mos.esante.gouv.fr/NOS/JDV_J01-XdsAuthorSpecialty-CISIS/FHIR/JDV-J01-XdsAuthorSpecialty-CISIS|20260928120000</t>
   </si>
 </sst>
 </file>

</xml_diff>